<commit_message>
Implement validated network CI/CD routing intent
</commit_message>
<xml_diff>
--- a/source_of_truth/network_source_of_truth.xlsx
+++ b/source_of_truth/network_source_of_truth.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Devices" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interfaces" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Links" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Desired_Config" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation_Rules" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Devices" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Interfaces" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Links" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Desired_Config" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Validation_Rules" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Devices'!$A$1:$H$4</definedName>
@@ -1325,7 +1325,7 @@
         </is>
       </c>
       <c r="E6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Enable EIGRP and RIP routing intent for R2 and R3
</commit_message>
<xml_diff>
--- a/source_of_truth/network_source_of_truth.xlsx
+++ b/source_of_truth/network_source_of_truth.xlsx
@@ -1415,7 +1415,7 @@
         </is>
       </c>
       <c r="E9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -1445,7 +1445,7 @@
         </is>
       </c>
       <c r="E10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -1505,7 +1505,7 @@
         </is>
       </c>
       <c r="E12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -1535,7 +1535,7 @@
         </is>
       </c>
       <c r="E13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>

</xml_diff>